<commit_message>
Soumission #119 : ZZ Test Hexatrust (à supprimer) [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$L$277</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$L$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L277"/>
+  <dimension ref="A1:L278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17760,8 +17760,70 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>ZZ Test Hexatrust (à supprimer)</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Entrée de test sur Hexatrust, sera supprimée juste après vérification.</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>test, chiffrement</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="F278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>Gestion des identités et des accès aux SI</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>https://zz-test-hexatrust.example</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>contact@zz-test-hexatrust.example</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>zz-test-hexatrust-a-supprimer.svg</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>zz-test-hexatrust-a-supprimer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L277"/>
+  <autoFilter ref="A1:L278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23018,7 +23080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J277"/>
+  <dimension ref="A1:J278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -36761,8 +36823,40 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>ZZ Test Hexatrust (à supprimer)</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="3" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr"/>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr"/>
+      <c r="J278" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J277"/>
+  <autoFilter ref="A1:J278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #120 : ZZ Test Hexatrust (à supprimer) [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -17768,12 +17768,12 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup / petite entreprise</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Entrée de test sur Hexatrust, sera supprimée juste après vérification.</t>
+          <t>Description modifiée sur Hexatrust via le formulaire de modification.</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17793,7 +17793,8 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
         </is>
       </c>
       <c r="H278" s="3" t="inlineStr">
@@ -36841,7 +36842,8 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
         </is>
       </c>
       <c r="E278" s="3" t="inlineStr"/>
@@ -36849,7 +36851,7 @@
       <c r="G278" s="3" t="inlineStr"/>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup / petite entreprise</t>
         </is>
       </c>
       <c r="I278" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Revert "Soumission #120 : ZZ Test Hexatrust (à supprimer) [approved]"
This reverts commit ae2849f27a50a2cc4b2d90e1fa39905f418cd1a0.
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -17768,12 +17768,12 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>Startup / petite entreprise</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Description modifiée sur Hexatrust via le formulaire de modification.</t>
+          <t>Entrée de test sur Hexatrust, sera supprimée juste après vérification.</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -17793,8 +17793,7 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
-PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
         </is>
       </c>
       <c r="H278" s="3" t="inlineStr">
@@ -36842,8 +36841,7 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
-PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
         </is>
       </c>
       <c r="E278" s="3" t="inlineStr"/>
@@ -36851,7 +36849,7 @@
       <c r="G278" s="3" t="inlineStr"/>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>Startup / petite entreprise</t>
+          <t>PME</t>
         </is>
       </c>
       <c r="I278" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Revert "Soumission #119 : ZZ Test Hexatrust (à supprimer) [approved]"
This reverts commit 3c174a610cd3dbc95d7be453654ebd47d5ca2fb5.
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$L$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$L$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L278"/>
+  <dimension ref="A1:L277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17760,70 +17760,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr">
-        <is>
-          <t>ZZ Test Hexatrust (à supprimer)</t>
-        </is>
-      </c>
-      <c r="B278" s="2" t="inlineStr">
-        <is>
-          <t>PME</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>Entrée de test sur Hexatrust, sera supprimée juste après vérification.</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>test, chiffrement</t>
-        </is>
-      </c>
-      <c r="E278" s="2" t="inlineStr">
-        <is>
-          <t>PR : Protéger</t>
-        </is>
-      </c>
-      <c r="F278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS : Sécurité des données</t>
-        </is>
-      </c>
-      <c r="G278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
-        </is>
-      </c>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>Gestion des identités et des accès aux SI</t>
-        </is>
-      </c>
-      <c r="I278" s="2" t="inlineStr">
-        <is>
-          <t>https://zz-test-hexatrust.example</t>
-        </is>
-      </c>
-      <c r="J278" s="2" t="inlineStr">
-        <is>
-          <t>contact@zz-test-hexatrust.example</t>
-        </is>
-      </c>
-      <c r="K278" s="2" t="inlineStr">
-        <is>
-          <t>zz-test-hexatrust-a-supprimer.svg</t>
-        </is>
-      </c>
-      <c r="L278" s="2" t="inlineStr">
-        <is>
-          <t>zz-test-hexatrust-a-supprimer</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L278"/>
+  <autoFilter ref="A1:L277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23080,7 +23018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J278"/>
+  <dimension ref="A1:J277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -36823,40 +36761,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="3" t="inlineStr">
-        <is>
-          <t>ZZ Test Hexatrust (à supprimer)</t>
-        </is>
-      </c>
-      <c r="B278" s="3" t="inlineStr">
-        <is>
-          <t>PR : Protéger</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS : Sécurité des données</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
-        </is>
-      </c>
-      <c r="E278" s="3" t="inlineStr"/>
-      <c r="F278" s="3" t="inlineStr"/>
-      <c r="G278" s="3" t="inlineStr"/>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>PME</t>
-        </is>
-      </c>
-      <c r="I278" s="3" t="inlineStr"/>
-      <c r="J278" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J278"/>
+  <autoFilter ref="A1:J277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data sync depuis Excel [auto]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solutions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listing référentiel NIST" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Référentiel NIST" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Solutions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Listing référentiel NIST" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Référentiel NIST" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>

</xml_diff>

<commit_message>
Soumission #122 : [TEST] Entreprise Hexatrust [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M277"/>
+  <dimension ref="A1:M278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19114,8 +19114,71 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>[TEST] Entreprise Hexatrust</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise de test Hexatrust, sera supprimée après vérification.</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>Contenu de test avec le mot hxfinalwitness pour valider l'indexation par le moteur de recherche.</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise des SI</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>https://test-hexatrust-final.example</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>contact@test-hexatrust-final.example</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>test-entreprise-hexatrust.svg</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>test-entreprise-hexatrust</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M277"/>
+  <autoFilter ref="A1:M278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24372,7 +24435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J277"/>
+  <dimension ref="A1:J278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38115,8 +38178,40 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>[TEST] Entreprise Hexatrust</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="3" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr"/>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr"/>
+      <c r="J278" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J277"/>
+  <autoFilter ref="A1:J278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #123 : [TEST] Entreprise Hexatrust [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -19122,12 +19122,12 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup / petite entreprise</t>
         </is>
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>Entreprise de test Hexatrust, sera supprimée après vérification.</t>
+          <t>Description courte modifiée sur Hexatrust.</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -19148,7 +19148,8 @@
       </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
         </is>
       </c>
       <c r="I278" s="3" t="inlineStr">
@@ -19158,7 +19159,7 @@
       </c>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>https://test-hexatrust-final.example</t>
+          <t>### Nouveau contact (si changement)</t>
         </is>
       </c>
       <c r="K278" s="2" t="inlineStr">
@@ -38196,7 +38197,8 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées</t>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
         </is>
       </c>
       <c r="E278" s="3" t="inlineStr"/>
@@ -38204,7 +38206,7 @@
       <c r="G278" s="3" t="inlineStr"/>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Startup / petite entreprise</t>
         </is>
       </c>
       <c r="I278" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Soumission #124 : [TEST] Entreprise Hexatrust [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19114,72 +19114,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr">
-        <is>
-          <t>[TEST] Entreprise Hexatrust</t>
-        </is>
-      </c>
-      <c r="B278" s="2" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>Description courte modifiée sur Hexatrust.</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>Contenu de test avec le mot hxfinalwitness pour valider l'indexation par le moteur de recherche.</t>
-        </is>
-      </c>
-      <c r="E278" s="3" t="inlineStr"/>
-      <c r="F278" s="2" t="inlineStr">
-        <is>
-          <t>PR : Protéger</t>
-        </is>
-      </c>
-      <c r="G278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS : Sécurité des données</t>
-        </is>
-      </c>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
-PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
-        </is>
-      </c>
-      <c r="I278" s="3" t="inlineStr">
-        <is>
-          <t>Maîtrise des SI</t>
-        </is>
-      </c>
-      <c r="J278" s="2" t="inlineStr">
-        <is>
-          <t>### Nouveau contact (si changement)</t>
-        </is>
-      </c>
-      <c r="K278" s="2" t="inlineStr">
-        <is>
-          <t>contact@test-hexatrust-final.example</t>
-        </is>
-      </c>
-      <c r="L278" s="2" t="inlineStr">
-        <is>
-          <t>test-entreprise-hexatrust.svg</t>
-        </is>
-      </c>
-      <c r="M278" s="2" t="inlineStr">
-        <is>
-          <t>test-entreprise-hexatrust</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M278"/>
+  <autoFilter ref="A1:M277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24436,7 +24372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J278"/>
+  <dimension ref="A1:J277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38179,41 +38115,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="3" t="inlineStr">
-        <is>
-          <t>[TEST] Entreprise Hexatrust</t>
-        </is>
-      </c>
-      <c r="B278" s="3" t="inlineStr">
-        <is>
-          <t>PR : Protéger</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS : Sécurité des données</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
-PR.DS-02 : La confidentialité, l'intégrité et la disponibilité des données en transit sont protégées</t>
-        </is>
-      </c>
-      <c r="E278" s="3" t="inlineStr"/>
-      <c r="F278" s="3" t="inlineStr"/>
-      <c r="G278" s="3" t="inlineStr"/>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="I278" s="3" t="inlineStr"/>
-      <c r="J278" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J278"/>
+  <autoFilter ref="A1:J277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #128 : Tacit [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M277"/>
+  <dimension ref="A1:M278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19114,8 +19114,73 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Tacit</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
+GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
+GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise des SI</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>https://tacit.now/</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>support@tacit.now</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>tacit.png</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>tacit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M277"/>
+  <autoFilter ref="A1:M278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24372,7 +24437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J277"/>
+  <dimension ref="A1:J278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38115,8 +38180,42 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
+GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
+GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="3" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr"/>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr"/>
+      <c r="J278" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J277"/>
+  <autoFilter ref="A1:J278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #129 : Tacit Trois N2 [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$279</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19179,8 +19179,75 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Tacit Trois N2</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr"/>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs
+ID.RA : Évaluation des risques</t>
+        </is>
+      </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
+GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
+GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise des SI</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>https://tacit.now/</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>support@tacit.now</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>tacit-trois-n2.png</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>tacit-trois-n2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M278"/>
+  <autoFilter ref="A1:M279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24437,7 +24504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J278"/>
+  <dimension ref="A1:J279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38214,8 +38281,44 @@
       <c r="I278" s="3" t="inlineStr"/>
       <c r="J278" s="3" t="inlineStr"/>
     </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>Tacit Trois N2</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs
+ID.RA : Évaluation des risques</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
+GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
+GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr"/>
+      <c r="F279" s="3" t="inlineStr"/>
+      <c r="G279" s="3" t="inlineStr"/>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr"/>
+      <c r="J279" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J278"/>
+  <autoFilter ref="A1:J279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #130 : Tacit [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$279</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M279"/>
+  <dimension ref="A1:M278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19117,7 +19117,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>Tacit</t>
+          <t>Tacit Trois N2</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -19143,7 +19143,9 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber</t>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs
+ID.RA : Évaluation des risques</t>
         </is>
       </c>
       <c r="H278" s="3" t="inlineStr">
@@ -19170,84 +19172,17 @@
       </c>
       <c r="L278" s="2" t="inlineStr">
         <is>
-          <t>tacit.png</t>
+          <t>tacit-trois-n2.png</t>
         </is>
       </c>
       <c r="M278" s="2" t="inlineStr">
         <is>
-          <t>tacit</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" s="2" t="inlineStr">
-        <is>
-          <t>Tacit Trois N2</t>
-        </is>
-      </c>
-      <c r="B279" s="2" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="C279" s="3" t="inlineStr">
-        <is>
-          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
-        </is>
-      </c>
-      <c r="D279" s="3" t="inlineStr">
-        <is>
-          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
-        </is>
-      </c>
-      <c r="E279" s="3" t="inlineStr"/>
-      <c r="F279" s="2" t="inlineStr">
-        <is>
-          <t>GV : Gouverner</t>
-        </is>
-      </c>
-      <c r="G279" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
-ID.AM : Gestion des actifs
-ID.RA : Évaluation des risques</t>
-        </is>
-      </c>
-      <c r="H279" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
-GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
-GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
-        </is>
-      </c>
-      <c r="I279" s="3" t="inlineStr">
-        <is>
-          <t>Maîtrise des SI</t>
-        </is>
-      </c>
-      <c r="J279" s="2" t="inlineStr">
-        <is>
-          <t>https://tacit.now/</t>
-        </is>
-      </c>
-      <c r="K279" s="2" t="inlineStr">
-        <is>
-          <t>support@tacit.now</t>
-        </is>
-      </c>
-      <c r="L279" s="2" t="inlineStr">
-        <is>
-          <t>tacit-trois-n2.png</t>
-        </is>
-      </c>
-      <c r="M279" s="2" t="inlineStr">
-        <is>
           <t>tacit-trois-n2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M279"/>
+  <autoFilter ref="A1:M278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24504,7 +24439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J279"/>
+  <dimension ref="A1:J278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38250,7 +38185,7 @@
     <row r="278">
       <c r="A278" s="3" t="inlineStr">
         <is>
-          <t>Tacit</t>
+          <t>Tacit Trois N2</t>
         </is>
       </c>
       <c r="B278" s="3" t="inlineStr">
@@ -38260,7 +38195,9 @@
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber</t>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs
+ID.RA : Évaluation des risques</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
@@ -38281,44 +38218,8 @@
       <c r="I278" s="3" t="inlineStr"/>
       <c r="J278" s="3" t="inlineStr"/>
     </row>
-    <row r="279">
-      <c r="A279" s="3" t="inlineStr">
-        <is>
-          <t>Tacit Trois N2</t>
-        </is>
-      </c>
-      <c r="B279" s="3" t="inlineStr">
-        <is>
-          <t>GV : Gouverner</t>
-        </is>
-      </c>
-      <c r="C279" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
-ID.AM : Gestion des actifs
-ID.RA : Évaluation des risques</t>
-        </is>
-      </c>
-      <c r="D279" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
-GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
-GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
-        </is>
-      </c>
-      <c r="E279" s="3" t="inlineStr"/>
-      <c r="F279" s="3" t="inlineStr"/>
-      <c r="G279" s="3" t="inlineStr"/>
-      <c r="H279" s="3" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="I279" s="3" t="inlineStr"/>
-      <c r="J279" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J279"/>
+  <autoFilter ref="A1:J278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #131 : Tacit Trois N2 [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19114,75 +19114,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr">
-        <is>
-          <t>Tacit Trois N2</t>
-        </is>
-      </c>
-      <c r="B278" s="2" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
-        </is>
-      </c>
-      <c r="E278" s="3" t="inlineStr"/>
-      <c r="F278" s="2" t="inlineStr">
-        <is>
-          <t>GV : Gouverner</t>
-        </is>
-      </c>
-      <c r="G278" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
-ID.AM : Gestion des actifs
-ID.RA : Évaluation des risques</t>
-        </is>
-      </c>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
-GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
-GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
-        </is>
-      </c>
-      <c r="I278" s="3" t="inlineStr">
-        <is>
-          <t>Maîtrise des SI</t>
-        </is>
-      </c>
-      <c r="J278" s="2" t="inlineStr">
-        <is>
-          <t>https://tacit.now/</t>
-        </is>
-      </c>
-      <c r="K278" s="2" t="inlineStr">
-        <is>
-          <t>support@tacit.now</t>
-        </is>
-      </c>
-      <c r="L278" s="2" t="inlineStr">
-        <is>
-          <t>tacit-trois-n2.png</t>
-        </is>
-      </c>
-      <c r="M278" s="2" t="inlineStr">
-        <is>
-          <t>tacit-trois-n2</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M278"/>
+  <autoFilter ref="A1:M277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24439,7 +24372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J278"/>
+  <dimension ref="A1:J277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38182,44 +38115,8 @@
         </is>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="3" t="inlineStr">
-        <is>
-          <t>Tacit Trois N2</t>
-        </is>
-      </c>
-      <c r="B278" s="3" t="inlineStr">
-        <is>
-          <t>GV : Gouverner</t>
-        </is>
-      </c>
-      <c r="C278" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
-ID.AM : Gestion des actifs
-ID.RA : Évaluation des risques</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis
-GV.SC-02 : Les rôles cyber des fournisseurs, clients et partenaires sont établis et coordonnés
-GV.SC-03 : La gestion des risques de la chaîne d'approvisionnement est intégrée à la gestion des risques cyber et d'entreprise</t>
-        </is>
-      </c>
-      <c r="E278" s="3" t="inlineStr"/>
-      <c r="F278" s="3" t="inlineStr"/>
-      <c r="G278" s="3" t="inlineStr"/>
-      <c r="H278" s="3" t="inlineStr">
-        <is>
-          <t>Startup / petite entreprise</t>
-        </is>
-      </c>
-      <c r="I278" s="3" t="inlineStr"/>
-      <c r="J278" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J278"/>
+  <autoFilter ref="A1:J277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #126 : Tacit [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$277</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M277"/>
+  <dimension ref="A1:M278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19114,8 +19114,72 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Tacit</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit est une plateforme SaaS de gestion de la sécurité produit pour les éditeurs logiciels. Tacit donne aux équipes sécurité des outils de preuve pour contrôler, trier avec contexte, coordonner les équipes, et démontrer leur posture sécuritaire à quiconque le demande, sur l'ensemble de leurs logiciels, durant tout leur cycle de vie produit.</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise des SI</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>https://tacit.now/</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>support@tacit.now</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>tacit.png</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>tacit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M277"/>
+  <autoFilter ref="A1:M278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24372,7 +24436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J277"/>
+  <dimension ref="A1:J278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38115,8 +38179,41 @@
         </is>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>Tacit</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>GV : Gouverner</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC : Gestion des risques de la chaîne d'approvisionnement cyber
+ID.AM : Gestion des actifs</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>GV.SC-01 : Un programme et une stratégie de gestion des risques de la chaîne d'approvisionnement cyber sont établis</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr"/>
+      <c r="F278" s="3" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr"/>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr"/>
+      <c r="J278" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J277"/>
+  <autoFilter ref="A1:J278"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #135 : NameShield [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -9917,7 +9917,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>ETI / scale-up</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -31458,7 +31458,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>ETI / scale-up</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Soumission #139 : Appaloosa [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$278</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$278</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$279</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19178,8 +19178,75 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Appaloosa</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>Appaloosa est une solution française hébergée sur un cloud SecNumCloud de Mobile Device Management (MDM/EMM) et de Mobile Application Management (MAM) pour iOS, Android, Windows et Mac. Elle permet aux entreprises de déployer, configurer et sécuriser leur flotte mobile en quelques minutes, sans toucher aux appareils.</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>Appaloosa simplifie la gestion de la mobilité d’entreprise. Notre plateforme SaaS permet aux équipes IT de piloter l’ensemble de leur flotte Apple, Android &amp; Windows depuis une console unique et intuitive.
+Grâce au zero-touch enrollment, les appareils sont préconfigurés dès leur mise en service : applications, Wi-Fi, messagerie et politiques de sécurité se déploient automatiquement. Notre Enterprise App Store intégré centralise la distribution des applications métier publiques, privées ou web avec mise à jour silencieuse à grande échelle.
+Appaloosa couvre les scénarios corporate-owned, BYOD et kiosk, et s’intègre avec votre suite de productivité et votre annuaire. Hébergée chez Outscale (qualifié SecNumCloud), la solution est opérationnelle en moins d’une journée.</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr"/>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>PR.PS : Sécurité des plateformes</t>
+        </is>
+      </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>PR.PS-01 : Les pratiques de gestion de configuration sont établies et appliquées
+PR.PS-02 : Les logiciels sont maintenus, remplacés et retirés en cohérence avec le risque
+PR.PS-05 : L'installation et l'exécution de logiciels non autorisés sont empêchées</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise de l'écosystème</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appaloosa.io</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>sales@appaloosa.io</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>appaloosa.svg</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>appaloosa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M278"/>
+  <autoFilter ref="A1:M279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24436,7 +24503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J278"/>
+  <dimension ref="A1:J279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38212,8 +38279,42 @@
       <c r="I278" s="3" t="inlineStr"/>
       <c r="J278" s="3" t="inlineStr"/>
     </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>Appaloosa</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>PR.PS : Sécurité des plateformes</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>PR.PS-01 : Les pratiques de gestion de configuration sont établies et appliquées
+PR.PS-02 : Les logiciels sont maintenus, remplacés et retirés en cohérence avec le risque
+PR.PS-05 : L'installation et l'exécution de logiciels non autorisés sont empêchées</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr"/>
+      <c r="F279" s="3" t="inlineStr"/>
+      <c r="G279" s="3" t="inlineStr"/>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr"/>
+      <c r="J279" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J278"/>
+  <autoFilter ref="A1:J279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #141 : Nuabee [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$279</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$280</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M279"/>
+  <dimension ref="A1:M280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19245,8 +19245,81 @@
         </is>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Nuabee</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>**Nuabee** est un éditeur français de solution de **[Plan de Reprise d'Activité](https://nuabee.fr/protection-pra-cloud/)** dans un Cloud public OpenStack. Il offre un _service managé de PRA_ incluant 3 classes de protection par serveur : backup étanche, backup avec tests automatique de redémarrage, PRA avec test semestriel.</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>Nuabee est un spécialiste français de la cyber-résilience, du PRA Cloud managé, du Disaster Recovery as a Service (DRaaS) et de la sauvegarde externalisée sécurisée pour les entreprises, ETI, collectivités et organisations multisites.
+Ses solutions couvrent la protection, la réplication, la restauration et le redémarrage des serveurs, machines virtuelles ou physiques, applications critiques et données, avec des objectifs de reprise RTO/RPO contractualisés.
+L’offre associe sauvegarde chiffrée, stockage immuable, Object Lock, isolation Air Gap, environnements Cloud de secours, supervision quotidienne et console de pilotage du Plan de Reprise d’Activité.
+Nuabee se différencie par une approche entièrement managée, des tests réguliers de restauration et de PRA, la modélisation du système d’information, l’automatisation des scénarios de reprise et l’accompagnement en situation de crise cyber.
+Les principaux cas d’usage sont la reprise après ransomware, cyberattaque, panne matérielle, sinistre informatique, indisponibilité d’un datacenter, corruption de données ou interruption d’activité.
+La solution contribue aux fonctions Protect, Respond et Recover du NIST CSF 2.0 et répond aux besoins de continuité d’activité, résilience opérationnelle, conformité, souveraineté des données et sécurisation des sauvegardes.</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr"/>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>RC : Récupérer</t>
+        </is>
+      </c>
+      <c r="G280" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP : Exécution du plan de reprise
+RS.MA : Gestion des incidents</t>
+        </is>
+      </c>
+      <c r="H280" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP-01 : La partie reprise du plan de réponse aux incidents est exécutée une fois déclenchée
+RC.RP-02 : Les actions de reprise sont sélectionnées, cadrées, priorisées et exécutées
+RC.RP-03 : L'intégrité des sauvegardes et autres actifs de restauration est vérifiée avant utilisation
+RC.RP-05 : L'intégrité des actifs restaurés est vérifiée et le retour à un état de fonctionnement normal est confirmé
+RC.RP-06 : La fin de la reprise d'incident est déclarée selon des critères, avec documentation complétée</t>
+        </is>
+      </c>
+      <c r="I280" s="3" t="inlineStr">
+        <is>
+          <t>Recensement des SI</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>https://nuabee.fr/</t>
+        </is>
+      </c>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>sales@nuabee.fr</t>
+        </is>
+      </c>
+      <c r="L280" s="2" t="inlineStr">
+        <is>
+          <t>nuabee.png</t>
+        </is>
+      </c>
+      <c r="M280" s="2" t="inlineStr">
+        <is>
+          <t>nuabee</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M279"/>
+  <autoFilter ref="A1:M280"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24503,7 +24576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J279"/>
+  <dimension ref="A1:J280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38313,8 +38386,45 @@
       <c r="I279" s="3" t="inlineStr"/>
       <c r="J279" s="3" t="inlineStr"/>
     </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>Nuabee</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>RC : Récupérer</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP : Exécution du plan de reprise
+RS.MA : Gestion des incidents</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>RC.RP-01 : La partie reprise du plan de réponse aux incidents est exécutée une fois déclenchée
+RC.RP-02 : Les actions de reprise sont sélectionnées, cadrées, priorisées et exécutées
+RC.RP-03 : L'intégrité des sauvegardes et autres actifs de restauration est vérifiée avant utilisation
+RC.RP-05 : L'intégrité des actifs restaurés est vérifiée et le retour à un état de fonctionnement normal est confirmé
+RC.RP-06 : La fin de la reprise d'incident est déclarée selon des critères, avec documentation complétée</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr"/>
+      <c r="F280" s="3" t="inlineStr"/>
+      <c r="G280" s="3" t="inlineStr"/>
+      <c r="H280" s="3" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="I280" s="3" t="inlineStr"/>
+      <c r="J280" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J279"/>
+  <autoFilter ref="A1:J280"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #142 : Cybee [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$280</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$281</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M280"/>
+  <dimension ref="A1:M281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19318,8 +19318,78 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>Cybee</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>**Cybee** est une plateforme européenne de sauvegarde Cloud cyber-résiliente qui protège les données et les systèmes grâce au chiffrement à la source, à l’immutabilité et à l’orchestration centralisée des politiques de sauvegarde. Elle est basée sur le moteur open source Restic.</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>Cybee est une plateforme européenne de sauvegarde Cloud cyber-résiliente destinée aux entreprises, ETI, collectivités, prestataires IT, infogéreurs et fournisseurs de services managés souhaitant sécuriser leurs données et systèmes critiques.
+Elle couvre la sauvegarde de fichiers, de serveurs Windows et Linux, de machines virtuelles et d’images système, ainsi que la restauration granulaire, planifiée ou bare-metal après une panne, une erreur humaine, une corruption de données ou une cyberattaque.
+La solution associe chiffrement à la source, contrôle d’intégrité cryptographique, stockage objet S3, sauvegardes immuables avec Object Lock, snapshots Restic, gestion des rétentions et séparation des clés et des environnements.
+Cybee se différencie par son orchestration centralisée, sa console de supervision, sa CMDB intégrée, la découverte automatique des actifs, la planification des politiques de protection et la traçabilité complète des opérations.
+Ses mécanismes d’authentification forte, de contrôle d’accès granulaire, de vérification des sauvegardes et de restauration rapide renforcent la protection contre les ransomwares et la résilience du système d’information.
+Les principaux cas d’usage sont la sauvegarde externalisée, la protection des données sensibles, la reprise après cyberattaque, la continuité d’activité, la modernisation d’architectures de backup et le déploiement d’une offre Backup as a Service souveraine. Elle s'appuie sur le moteur de sauvegarde open source Restic.</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr"/>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données
+PR.IR : Résilience de l'infrastructure technologique</t>
+        </is>
+      </c>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-11 : Les sauvegardes de données sont créées, protégées, maintenues et testées</t>
+        </is>
+      </c>
+      <c r="I281" s="3" t="inlineStr">
+        <is>
+          <t>Recensement des SI</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>https://cybee.fr/</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>https://cybee.fr/contact/</t>
+        </is>
+      </c>
+      <c r="L281" s="2" t="inlineStr">
+        <is>
+          <t>cybee.png</t>
+        </is>
+      </c>
+      <c r="M281" s="2" t="inlineStr">
+        <is>
+          <t>cybee</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M280"/>
+  <autoFilter ref="A1:M281"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24576,7 +24646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J280"/>
+  <dimension ref="A1:J281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38423,8 +38493,42 @@
       <c r="I280" s="3" t="inlineStr"/>
       <c r="J280" s="3" t="inlineStr"/>
     </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>Cybee</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>PR : Protéger</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS : Sécurité des données
+PR.IR : Résilience de l'infrastructure technologique</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>PR.DS-01 : La confidentialité, l'intégrité et la disponibilité des données au repos sont protégées
+PR.DS-11 : Les sauvegardes de données sont créées, protégées, maintenues et testées</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr"/>
+      <c r="F281" s="3" t="inlineStr"/>
+      <c r="G281" s="3" t="inlineStr"/>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I281" s="3" t="inlineStr"/>
+      <c r="J281" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J280"/>
+  <autoFilter ref="A1:J281"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #143 : Snowpack [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -15040,7 +15040,8 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Snowpack a conçu une technologie de réseau privé invisible baptisée VIPN qui fragmente et anonymise les communications pour masquer utilisateurs, services et infrastructures. Le catalogue regroupe Invisible Access pour la navigation anonyme, Invisible Services, Invisible Infra et des SDK/API Invisible by Snowpack. La société par actions simplifiée a son siège à Orsay (RCS Evry 900 526 716) et travaille avec le CEA et Bpifrance.</t>
+          <t>**Fournisseur de connectivité furtive, sécurisée et résiliente.** 
+Grâce à notre technologie brevetée VIPN (_Virtual &amp; Invisible Private Network_), réduisez et protégez votre surface d’attaque externe en ne faisant confiance à personne: rendez **invisibles** vos assets numériques sensibles exposés sur Internet et protégez vos utilisateurs, services et infrastructures des cyberattaques.</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -15086,7 +15087,7 @@
       </c>
       <c r="L217" s="2" t="inlineStr">
         <is>
-          <t>Snowpack_01.png</t>
+          <t>snowpack.png</t>
         </is>
       </c>
       <c r="M217" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Soumission #144 : Cyberlib [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$281</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$282</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$282</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M281"/>
+  <dimension ref="A1:M282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19389,8 +19389,81 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Cyberlib</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Cyberlib est une plateforme SaaS / On-Premise permet de gérer le durcissement de configuration (Hardening) des systèmes durablement et à l'échelle d'un système d'information d'entreprise. Elle permet de gérer tout le cycle de vie du Hardening d'un système (audit - déploiement - supervision continue) pour réduire efficacement la surface d'attaque et colmater les brèches en réponse à des incidents de sécurité.</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>Cyberlib est une plateforme SaaS B2B de cybersécurité spécialisée dans le durcissement natif des endpoints (hardening), avec une approche réactive et préventive visant à réduire la surface d'attaque en appliquant des politiques de durcissement cohérentes et auditées avant/après la survenue des incidents. Éditée et opérée par la société Cyberlib, la solution est 100 % française (conception, hébergement, maintenance) et hébergée en cloud de confiance qualifié SecNumCloud 3.2. Elle se compose d'une application Web (console d'administration centralisée) et d'un connecteur "agentless" avec solution tierce compatible disposant d'agents installés sur les endpoints du SI (Intune, JAMF, XDR type HarfanfLab/Crowstrike...) et/ou d'un agent logiciel léger à installer sur les postes et serveurs à durcir, disponible en mode SaaS mutualisé, en instance dédiée ou en déploiement On-Premise / souverain chez le client pour les environnements les plus sensibles, cloisonnés, air-gapped ou soumis à des contraintes de localisation de données. Le cœur de l'offre repose sur la gestion bout en bout du durcissement de configuration : paramétrage et déploiement sans script de plus de 1600 politiques de sécurité natives du système d'exploitation, création de référentiels de sécurité en mode no-code, création de groupes de postes et automatisation du déploiement des règles de durcissement sur l'ensemble des endpoints concernés (logique similaire aux GPO), le tout utilisable avec ou sans Active Directory. Mots-clés associés : hardening, durcissement, configuration hardening, security baseline, benchmark de sécurité, gestion de configuration, posture management, endpoint hardening, server hardening, OS hardening, no-code, sans script, agent léger, console web, GPO, Active Directory, MDM, Intune, PowerShell, Windows, macOS, Linux. 
+Sur le plan fonctionnel, Cyberlib couvre l'inventaire et la visualisation du niveau de durcissement du parc, la définition de référentiels et de politiques, le déploiement automatisé, le contrôle continu de la dérive de configuration, la remédiation et le reporting de conformité. La solution assure la maîtrise des endpoints et des serveurs, y compris le shadow IT hors Active Directory, les postes et machines projet et les systèmes industriels, pour une gouvernance complète : visualisation, durcissement et pilotage centralisé ; elle protège les terminaux même hors réseau, en mobilité ou en shadow IT, sans surcharge pour les équipes internes. L'agent se déploie de façon automatisée via une commande de type PowerShell, à travers l'AD ou le MDM existant, avec une gestion dynamique de charge pour des milliers d'agents et une architecture multi-zone redondée en actif-actif. Cyberlib s'intègre aux environnements existants et se positionne en amont des outils de type EDR, XDR et SIEM, en améliorant l'hygiène de sécurité et la résistance des postes ; elle s'adresse aux MSP et MSSP comme aux organisations souhaitant industrialiser le hardening sans alourdir l'exploitation. Mots-clés associés : réduction de la surface d'attaque, attack surface reduction, Zero Trust, moindre privilège, durcissement automatisé, remédiation continue, dérive de configuration, drift, shadow IT, OT/ICS, parc hétérogène, EDR, XDR, SIEM, MSP, MSSP, infogérance, ESN, cabinets de conseil, industrie, logistique, services, chiffrement, sauvegarde anti-ransomware, rançongiciel, sensibilisation, RGPD. 
+Cyberlib adresse les organisations mid-Market et Grand groupe : PME, ETI, grands comptes, groupes multi-filiales et collectivités — avec une logique d'industrialisation de la gestion de surface d'attaque et/ou de la conformité réglementaire. La plateforme apporte un alignement CIS, NIST, ISO 27001 et RGPD, des tableaux de bord centralisés et des rapports exportables pour les audits internes et externes, ainsi qu'une interface intuitive de suivi du niveau de durcissement, un support à la gestion des effets de bord en cas d'anomalie critique, un accompagnement personnalisé (paramétrage sur-mesure, intégration au SI, assistance premium) et des ateliers avec des consultants seniors. Elle répond aux exigences de RGPD, NIS2, ISO 27001, ANSSI, PCI-DSS et HIPAA. Côté souveraineté et confiance : solution souveraine opérée et hébergée en France, dans des infrastructures ISO 27001 et HDS et SecNumCloud / Cloud de confiance. La solution est reconnue par l'écosystème : Lauréat Innov'Up de la Région Île-de-France et Bpifrance, Trophée Cybernight et Trophée de l'innovation du Cybershow Paris catégorie Start-up. Mots-clés associés : cybersécurité souveraine, French Tech, made in France, Cloud de confiance, hébergement France, ISO 27001, HDS, ANSSI, CIS Benchmarks, NIST CSF, NIS2, DORA, RGPD, PCI-DSS, HIPAA, SOX, conformité, audit, preuve de conformité, gouvernance, gestion des risques, résilience cyber, continuité d'activité, licence par poste, abonnement, SaaS, On-Premise, hybride. Cyberlib est également disponible sur les marchés publics (UGAP, CANUT, CAIH, ...)</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr"/>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>PR.IR : Résilience de l'infrastructure technologique
+RS.MI : Atténuation des incidents
+GV.OV : Supervision</t>
+        </is>
+      </c>
+      <c r="H282" s="3" t="inlineStr">
+        <is>
+          <t>GV.OV-03 : La performance de la gestion des risques cyber est évaluée et revue pour ajustement
+PR.IR-03 : Des mécanismes sont mis en œuvre pour atteindre les exigences de résilience en situation normale et adverse
+PR.IR-01 : Les réseaux et environnements sont protégés contre les accès et usages logiques non autorisés
+PR.IR-04 : Une capacité de ressources adéquate pour assurer la disponibilité est maintenue
+PR.IR-02 : Les actifs technologiques de l'organisation sont protégés contre les menaces environnementales
+RS.MI-01 : Les incidents sont confinés
+RS.MI-02 : Les incidents sont éradiqués</t>
+        </is>
+      </c>
+      <c r="I282" s="3" t="inlineStr">
+        <is>
+          <t>Sécurisation de l'architecture des SI</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>https://cyberlib.io</t>
+        </is>
+      </c>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>contact@cyberlib.io</t>
+        </is>
+      </c>
+      <c r="L282" s="2" t="inlineStr">
+        <is>
+          <t>cyberlib.png</t>
+        </is>
+      </c>
+      <c r="M282" s="2" t="inlineStr">
+        <is>
+          <t>cyberlib</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M281"/>
+  <autoFilter ref="A1:M282"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24647,7 +24720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J281"/>
+  <dimension ref="A1:J282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38528,8 +38601,48 @@
       <c r="I281" s="3" t="inlineStr"/>
       <c r="J281" s="3" t="inlineStr"/>
     </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>Cyberlib</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>PR.IR : Résilience de l'infrastructure technologique
+RS.MI : Atténuation des incidents
+GV.OV : Supervision</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>GV.OV-03 : La performance de la gestion des risques cyber est évaluée et revue pour ajustement
+PR.IR-03 : Des mécanismes sont mis en œuvre pour atteindre les exigences de résilience en situation normale et adverse
+PR.IR-01 : Les réseaux et environnements sont protégés contre les accès et usages logiques non autorisés
+PR.IR-04 : Une capacité de ressources adéquate pour assurer la disponibilité est maintenue
+PR.IR-02 : Les actifs technologiques de l'organisation sont protégés contre les menaces environnementales
+RS.MI-01 : Les incidents sont confinés
+RS.MI-02 : Les incidents sont éradiqués</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr"/>
+      <c r="F282" s="3" t="inlineStr"/>
+      <c r="G282" s="3" t="inlineStr"/>
+      <c r="H282" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I282" s="3" t="inlineStr"/>
+      <c r="J282" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J281"/>
+  <autoFilter ref="A1:J282"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #146 : CHEOPS TECHNOLOGY [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$282</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$282</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$283</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M282"/>
+  <dimension ref="A1:M283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19462,8 +19462,84 @@
         </is>
       </c>
     </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>CHEOPS TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>ETI / scale-up</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>CHEOPS TECHNOLOGY, expert en infrastructures informatiques sécurisées depuis 1998 en France et en Suisse, opère via sa division Cyberdéfense la solution CyberPatriot® : détection et réponse managée (SOC/MDR) 24/7 depuis la France et la Suisse, avec 2 SOC, 2 CSIRT et 1 CERT certifié ISO 27001/27035 membre du FIRST.
+CyberPatriot® repose sur un socle open source et intègre nativement une IA privée, hébergée et opérée en interne, aucune donnée client ne sort de la plateforme, garantissant souveraineté, transparence et réversibilité, en approche multi-éditeurs.</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>CHEOPS TECHNOLOGY est un groupe français expert en infrastructures informatiques sécurisées depuis 1998, l'un des leaders du Cloud Computing et de la Cybersécurité en France et en Suisse : 750 collaborateurs, plus de 2 000 clients, 14 agences et 8 datacenters souverains. Ses quatre métiers : Cloud &amp; Services Managés (cloud privé, public, hybride, hébergement souverain, infogérance, SLA et réversibilité), Cyberdéfense, Infrastructure (serveurs, stockage, sauvegarde, réseau) et Modernisation Technologique (cloud native, Factory Applicative, Factory IA).
+Sa division CHEOPS CYBERDÉFENSE, une soixantaine d'experts certifiés (OSCP, GIAC, CISSP, CEH, etc.), opère CyberPatriot®, sa solution de SOC managé / MDR capitalisant sur plus de 10 ans d'expérience en supervision de sécurité : détection et réponse 24/7, threat intelligence, avec 2 SOC, 2 CSIRT et 1 CERT certifié ISO 27001/27035 membre du FIRST, plus de 10 milliards d'événements analysés par jour. CyberPatriot® combine expertise offensive et défensive, processus conformes aux normes internationales (ISO 27001, ISO 27035, NIST SP 800-61) et technologies fondées sur les modèles « SOC as Code » et « Detection as Code ». Multi-éditeurs et adapté aux environnements on-premise, cloud privé ou public, il garantit un hébergement des données selon les exigences de souveraineté du client, en France ou en Suisse. En cas d'incident majeur, les équipes SOC, CSIRT et CERT interviennent de manière coordonnée, jusqu'à la gestion de crise.
+Services : audit de sécurité, test d'intrusion (pentest), red team, évaluation de maturité, OSINT, fuite de données, phishing et sensibilisation, gestion des vulnérabilités, sécurité managée EDR, XDR, SIEM, SOAR, WAF, PAM, ZTNA, réponse à incident, forensic, gestion de crise ransomware, et GRC : PSSI, analyse de risques, RSSI as a Service, conformité ISO 27001, NIS2, DORA, RGPD, NIST CSF. Portail client SOC Gold : cockpit temps réel multi-éditeurs (alertes, investigations, maturité, veille CVE/PSIRT).
+Stack technologique : la plateforme de détection et de réponse CyberPatriot® est construite sur un socle de solutions open source éprouvées et maîtrisées par nos équipes. Elastic (SIEM/détection), MISP (partage de renseignement sur la menace), IRIS (réponse à incident), garantissant transparence, auditabilité, réversibilité et indépendance technologique, dans une logique « SOC as Code » et « Detection as Code » (Caldera, Atomic Redteam, Mythic C2, RTA). Ce socle s'appuie sur des solutions souveraines françaises et européennes (Wallix, Stormshield, Check Point, WithSecure) et s'interface avec les principales technologies EDR/XDR du marché opérées chez nos clients (CrowdStrike, SentinelOne, HarfangLab, Trend Micro, Microsoft Defender), dans une approche multi-éditeurs sans dépendance à un fournisseur unique.
+Certifications groupe : ISO 27001, ISO 20000-1, HDS v2, ISAE 3402 Type 2, hébergement souverain en France et en Suisse.
+Cibles : ETI, PME, grands comptes, secteur public, santé, industrie, banque-assurance, en France et en Suisse.</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr"/>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>DE : Détecter</t>
+        </is>
+      </c>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>DE.CM : Surveillance continue
+RS.AN : Analyse des incidents
+RS.MA : Gestion des incidents</t>
+        </is>
+      </c>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>DE.CM-06 : Les activités et services des prestataires externes sont surveillés pour détecter les événements indésirables
+DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables
+RS.AN-03 : Une analyse est menée pour établir ce qui s'est passé et la cause racine de l'incident
+RS.AN-06 : Les actions menées durant une investigation sont enregistrées avec intégrité et provenance
+DE.CM-03 : L'activité du personnel et l'usage des technologies sont surveillés pour détecter les événements indésirables
+RS.AN-08 : L'ampleur d'un incident est estimée et validée</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr">
+        <is>
+          <t>Identification et réaction aux incidents de sécurité</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cheops-technology.com/</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>contact@cheops.fr</t>
+        </is>
+      </c>
+      <c r="L283" s="2" t="inlineStr">
+        <is>
+          <t>cheops-technology.png</t>
+        </is>
+      </c>
+      <c r="M283" s="2" t="inlineStr">
+        <is>
+          <t>cheops-technology</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M282"/>
+  <autoFilter ref="A1:M283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24720,7 +24796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J282"/>
+  <dimension ref="A1:J283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38641,8 +38717,47 @@
       <c r="I282" s="3" t="inlineStr"/>
       <c r="J282" s="3" t="inlineStr"/>
     </row>
+    <row r="283">
+      <c r="A283" s="3" t="inlineStr">
+        <is>
+          <t>CHEOPS TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>DE : Détecter</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>DE.CM : Surveillance continue
+RS.AN : Analyse des incidents
+RS.MA : Gestion des incidents</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>DE.CM-06 : Les activités et services des prestataires externes sont surveillés pour détecter les événements indésirables
+DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables
+RS.AN-03 : Une analyse est menée pour établir ce qui s'est passé et la cause racine de l'incident
+RS.AN-06 : Les actions menées durant une investigation sont enregistrées avec intégrité et provenance
+DE.CM-03 : L'activité du personnel et l'usage des technologies sont surveillés pour détecter les événements indésirables
+RS.AN-08 : L'ampleur d'un incident est estimée et validée</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr"/>
+      <c r="F283" s="3" t="inlineStr"/>
+      <c r="G283" s="3" t="inlineStr"/>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>ETI / scale-up</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr"/>
+      <c r="J283" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J282"/>
+  <autoFilter ref="A1:J283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #147 : SecMate [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$283</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$284</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M283"/>
+  <dimension ref="A1:M284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19538,8 +19538,78 @@
         </is>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>SecMate</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>SecMate aide les fabricants de produits critiques à savoir si leur logiciel peut être livré en toute sécurité. La plateforme identifie les vulnérabilités réellement exploitables et transforme les alertes existantes en décisions claires.</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>SecMate est une plateforme de décision pour la sécurité des produits. Elle aide les fabricants à déterminer si une version peut être livrée en toute sécurité.
+Son moteur propriétaire rassemble le code source, les dépendances, la documentation, la configuration, le modèle de menaces et les résultats des outils existants. Il recherche les vulnérabilités inconnues et les failles métier, puis évalue leur exploitabilité et leur impact dans le contexte réel du produit.
+SecMate transforme ainsi un grand nombre de signaux techniques en quelques risques concrets. À chaque version, la plateforme fournit une décision claire : corriger, accepter ou bloquer. Cette décision peut être intégrée à la chaîne de développement comme contrôle avant livraison.
+SecMate s’adresse aux fabricants de produits numériques, en particulier dans les environnements critiques ou réglementés. La plateforme accompagne leurs démarches de sécurité produit, de conformité et de mise sur le marché. Les principaux cas d’usage sont la découverte et la validation de vulnérabilités, l’analyse des chemins d’attaque, la modélisation des menaces, la priorisation des corrections et la décision de livraison. Le moteur de SecMate a déjà découvert plus de 100 vulnérabilités inconnues dans des logiciels embarqués et critiques.
+SecMate est disponible sous forme de service hébergé, dans un réseau privé, sur l’infrastructure du client ou dans un environnement isolé.</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr"/>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>ID : Identifier</t>
+        </is>
+      </c>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA : Évaluation des risques
+PR.PS : Sécurité des plateformes</t>
+        </is>
+      </c>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA-01 : Les vulnérabilités des actifs sont identifiées, validées et enregistrées
+ID.RA-04 : Les impacts et probabilités potentiels des menaces exploitant les vulnérabilités sont enregistrés
+ID.RA-05 : Menaces, vulnérabilités, probabilités et impacts informent le risque inhérent et la priorisation</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr">
+        <is>
+          <t>Mise en œuvre d'une approche par les risques</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>https://secmate.dev</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>contact@secmate.dev</t>
+        </is>
+      </c>
+      <c r="L284" s="2" t="inlineStr">
+        <is>
+          <t>secmate.svg</t>
+        </is>
+      </c>
+      <c r="M284" s="2" t="inlineStr">
+        <is>
+          <t>secmate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M283"/>
+  <autoFilter ref="A1:M284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24796,7 +24866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38756,8 +38826,43 @@
       <c r="I283" s="3" t="inlineStr"/>
       <c r="J283" s="3" t="inlineStr"/>
     </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>SecMate</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>ID : Identifier</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA : Évaluation des risques
+PR.PS : Sécurité des plateformes</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA-01 : Les vulnérabilités des actifs sont identifiées, validées et enregistrées
+ID.RA-04 : Les impacts et probabilités potentiels des menaces exploitant les vulnérabilités sont enregistrés
+ID.RA-05 : Menaces, vulnérabilités, probabilités et impacts informent le risque inhérent et la priorisation</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr"/>
+      <c r="F284" s="3" t="inlineStr"/>
+      <c r="G284" s="3" t="inlineStr"/>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>Startup / petite entreprise</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr"/>
+      <c r="J284" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J283"/>
+  <autoFilter ref="A1:J284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Logo Mailinblack (Protect) : le logo officiel a la place du pictogramme
L'ancien fichier etait un pictogramme SVG de 32x29 (le bouclier seul, sans le nom). Remplace par le
logo complet publie sur mailinblack.com (PNG 400x80). Excel et solutions.json mis a jour.
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Solutions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Listing référentiel NIST" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Référentiel NIST" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solutions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listing référentiel NIST" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Référentiel NIST" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$284</definedName>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
-          <t>Mailinblack (Protect)_svg.svg</t>
+          <t>Mailinblack (Protect)_01.png</t>
         </is>
       </c>
       <c r="M132" s="2" t="inlineStr">
@@ -22043,12 +22043,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22066,12 +22060,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22089,12 +22077,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22112,12 +22094,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22135,9 +22111,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -22170,12 +22143,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22193,12 +22160,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22216,12 +22177,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22239,12 +22194,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22262,12 +22211,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22285,12 +22228,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22308,9 +22245,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -22343,12 +22277,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22366,12 +22294,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22389,12 +22311,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22412,9 +22328,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -22447,12 +22360,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22470,9 +22377,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -22505,12 +22409,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22528,12 +22426,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22551,9 +22443,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
       <c r="D23" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -22586,12 +22475,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22609,12 +22492,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22632,12 +22509,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22655,12 +22526,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22678,12 +22543,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22701,12 +22560,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22724,12 +22577,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22747,12 +22594,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22770,12 +22611,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22840,12 +22675,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22863,12 +22692,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22886,12 +22709,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22909,12 +22726,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22932,12 +22743,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22955,12 +22760,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -22978,9 +22777,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
       <c r="D40" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23013,12 +22809,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23036,12 +22826,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23059,12 +22843,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23082,12 +22860,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23105,12 +22877,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23128,12 +22894,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n"/>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23151,12 +22911,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23174,12 +22928,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23197,12 +22945,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23220,9 +22962,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23255,12 +22994,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23278,12 +23011,6 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="n"/>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23301,12 +23028,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23371,12 +23092,6 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23394,12 +23109,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23417,12 +23126,6 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23440,12 +23143,6 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23463,12 +23160,6 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23486,9 +23177,6 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="n"/>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="n"/>
       <c r="D60" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23521,12 +23209,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23544,9 +23226,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="n"/>
-      <c r="B62" s="4" t="n"/>
-      <c r="C62" s="4" t="n"/>
       <c r="D62" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23579,12 +23258,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23602,12 +23275,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n"/>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23625,12 +23292,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
-      <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23648,9 +23309,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="n"/>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
       <c r="D66" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23683,12 +23341,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="n"/>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="4" t="n"/>
-      <c r="E67" s="4" t="n"/>
-      <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23706,12 +23358,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="n"/>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="n"/>
-      <c r="F68" s="4" t="n"/>
       <c r="G68" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23729,12 +23375,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="n"/>
-      <c r="B69" s="4" t="n"/>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="4" t="n"/>
-      <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23752,12 +23392,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="4" t="n"/>
-      <c r="B70" s="4" t="n"/>
-      <c r="C70" s="4" t="n"/>
-      <c r="D70" s="4" t="n"/>
-      <c r="E70" s="4" t="n"/>
-      <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23775,12 +23409,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="n"/>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="n"/>
       <c r="G71" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23798,9 +23426,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="n"/>
-      <c r="B72" s="4" t="n"/>
-      <c r="C72" s="4" t="n"/>
       <c r="D72" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -23833,12 +23458,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="n"/>
-      <c r="B73" s="4" t="n"/>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
-      <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23856,12 +23475,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="n"/>
-      <c r="B74" s="4" t="n"/>
-      <c r="C74" s="4" t="n"/>
-      <c r="D74" s="4" t="n"/>
-      <c r="E74" s="4" t="n"/>
-      <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23879,12 +23492,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="n"/>
-      <c r="B75" s="4" t="n"/>
-      <c r="C75" s="4" t="n"/>
-      <c r="D75" s="4" t="n"/>
-      <c r="E75" s="4" t="n"/>
-      <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23949,12 +23556,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="n"/>
-      <c r="B77" s="4" t="n"/>
-      <c r="C77" s="4" t="n"/>
-      <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="n"/>
-      <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23972,12 +23573,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="n"/>
-      <c r="B78" s="4" t="n"/>
-      <c r="C78" s="4" t="n"/>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="4" t="n"/>
-      <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -23995,12 +23590,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="4" t="n"/>
-      <c r="B79" s="4" t="n"/>
-      <c r="C79" s="4" t="n"/>
-      <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="n"/>
-      <c r="F79" s="4" t="n"/>
       <c r="G79" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24018,12 +23607,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="n"/>
-      <c r="B80" s="4" t="n"/>
-      <c r="C80" s="4" t="n"/>
-      <c r="D80" s="4" t="n"/>
-      <c r="E80" s="4" t="n"/>
-      <c r="F80" s="4" t="n"/>
       <c r="G80" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24041,9 +23624,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="n"/>
-      <c r="B81" s="4" t="n"/>
-      <c r="C81" s="4" t="n"/>
       <c r="D81" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -24076,12 +23656,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="n"/>
-      <c r="B82" s="4" t="n"/>
-      <c r="C82" s="4" t="n"/>
-      <c r="D82" s="4" t="n"/>
-      <c r="E82" s="4" t="n"/>
-      <c r="F82" s="4" t="n"/>
       <c r="G82" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24099,12 +23673,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="n"/>
-      <c r="B83" s="4" t="n"/>
-      <c r="C83" s="4" t="n"/>
-      <c r="D83" s="4" t="n"/>
-      <c r="E83" s="4" t="n"/>
-      <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24122,12 +23690,6 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="n"/>
-      <c r="B84" s="4" t="n"/>
-      <c r="C84" s="4" t="n"/>
-      <c r="D84" s="4" t="n"/>
-      <c r="E84" s="4" t="n"/>
-      <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24145,12 +23707,6 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="n"/>
-      <c r="B85" s="4" t="n"/>
-      <c r="C85" s="4" t="n"/>
-      <c r="D85" s="4" t="n"/>
-      <c r="E85" s="4" t="n"/>
-      <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24168,12 +23724,6 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="4" t="n"/>
-      <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="n"/>
-      <c r="D86" s="4" t="n"/>
-      <c r="E86" s="4" t="n"/>
-      <c r="F86" s="4" t="n"/>
       <c r="G86" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24238,12 +23788,6 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="n"/>
-      <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="n"/>
-      <c r="D88" s="4" t="n"/>
-      <c r="E88" s="4" t="n"/>
-      <c r="F88" s="4" t="n"/>
       <c r="G88" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24261,12 +23805,6 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="n"/>
-      <c r="B89" s="4" t="n"/>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="4" t="n"/>
-      <c r="E89" s="4" t="n"/>
-      <c r="F89" s="4" t="n"/>
       <c r="G89" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24284,12 +23822,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="n"/>
-      <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
-      <c r="E90" s="4" t="n"/>
-      <c r="F90" s="4" t="n"/>
       <c r="G90" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24307,12 +23839,6 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="n"/>
-      <c r="B91" s="4" t="n"/>
-      <c r="C91" s="4" t="n"/>
-      <c r="D91" s="4" t="n"/>
-      <c r="E91" s="4" t="n"/>
-      <c r="F91" s="4" t="n"/>
       <c r="G91" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24330,9 +23856,6 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="4" t="n"/>
-      <c r="B92" s="4" t="n"/>
-      <c r="C92" s="4" t="n"/>
       <c r="D92" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -24365,12 +23888,6 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="n"/>
-      <c r="B93" s="4" t="n"/>
-      <c r="C93" s="4" t="n"/>
-      <c r="D93" s="4" t="n"/>
-      <c r="E93" s="4" t="n"/>
-      <c r="F93" s="4" t="n"/>
       <c r="G93" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24388,12 +23905,6 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="n"/>
-      <c r="B94" s="4" t="n"/>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="4" t="n"/>
-      <c r="E94" s="4" t="n"/>
-      <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24411,12 +23922,6 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="n"/>
-      <c r="B95" s="4" t="n"/>
-      <c r="C95" s="4" t="n"/>
-      <c r="D95" s="4" t="n"/>
-      <c r="E95" s="4" t="n"/>
-      <c r="F95" s="4" t="n"/>
       <c r="G95" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24434,9 +23939,6 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="n"/>
-      <c r="B96" s="4" t="n"/>
-      <c r="C96" s="4" t="n"/>
       <c r="D96" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -24469,12 +23971,6 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="n"/>
-      <c r="B97" s="4" t="n"/>
-      <c r="C97" s="4" t="n"/>
-      <c r="D97" s="4" t="n"/>
-      <c r="E97" s="4" t="n"/>
-      <c r="F97" s="4" t="n"/>
       <c r="G97" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24492,9 +23988,6 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="n"/>
-      <c r="B98" s="4" t="n"/>
-      <c r="C98" s="4" t="n"/>
       <c r="D98" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -24527,12 +24020,6 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="n"/>
-      <c r="B99" s="4" t="n"/>
-      <c r="C99" s="4" t="n"/>
-      <c r="D99" s="4" t="n"/>
-      <c r="E99" s="4" t="n"/>
-      <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24597,12 +24084,6 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="n"/>
-      <c r="B101" s="4" t="n"/>
-      <c r="C101" s="4" t="n"/>
-      <c r="D101" s="4" t="n"/>
-      <c r="E101" s="4" t="n"/>
-      <c r="F101" s="4" t="n"/>
       <c r="G101" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24620,12 +24101,6 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="n"/>
-      <c r="B102" s="4" t="n"/>
-      <c r="C102" s="4" t="n"/>
-      <c r="D102" s="4" t="n"/>
-      <c r="E102" s="4" t="n"/>
-      <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24643,12 +24118,6 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="n"/>
-      <c r="B103" s="4" t="n"/>
-      <c r="C103" s="4" t="n"/>
-      <c r="D103" s="4" t="n"/>
-      <c r="E103" s="4" t="n"/>
-      <c r="F103" s="4" t="n"/>
       <c r="G103" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24666,12 +24135,6 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="4" t="n"/>
-      <c r="B104" s="4" t="n"/>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24689,12 +24152,6 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="4" t="n"/>
-      <c r="B105" s="4" t="n"/>
-      <c r="C105" s="4" t="n"/>
-      <c r="D105" s="4" t="n"/>
-      <c r="E105" s="4" t="n"/>
-      <c r="F105" s="4" t="n"/>
       <c r="G105" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>
@@ -24712,9 +24169,6 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="n"/>
-      <c r="B106" s="4" t="n"/>
-      <c r="C106" s="4" t="n"/>
       <c r="D106" s="4" t="inlineStr">
         <is>
           <t>NIST 2</t>
@@ -24747,12 +24201,6 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="4" t="n"/>
-      <c r="B107" s="4" t="n"/>
-      <c r="C107" s="4" t="n"/>
-      <c r="D107" s="4" t="n"/>
-      <c r="E107" s="4" t="n"/>
-      <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="inlineStr">
         <is>
           <t>NIST 3</t>

</xml_diff>

<commit_message>
Soumission #138 : F24 [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$284</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$285</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$285</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M284"/>
+  <dimension ref="A1:M285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19608,8 +19608,78 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Grand groupe</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>F24 propose une suite de résilience de bout en bout.
+Solution en mode SaaS, F24 garanti un environnement sécurisé, hautement disponible et répond à vos besoins de communication d'urgence, de mobilisation de cellule de crise de gestion d'incident, intégrant une main courante, un Chat, une visioconférence, une solution de GRC, BIA et la possibilité de générer vos Retex. 
+F24 propose une version d'exercice afin de tester vos plans d'actions.</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>Nos solutions couvrent l'ensemble de la chaîne de la résilience organisationnelle, depuis la Threat Intelligence, la GRC (Gouvernance, Risques et Conformité) et les Business Impact Analyses (BIA), jusqu'à l'alerte fonctionnelle ou l'alerte de masse et la mobilisation des équipes de crise. Elles permettent également de piloter la gestion de crise et des événements, d'assurer une main courante automatisée, de capitaliser sur les retours d'expérience (RETEX) et de gérer efficacement les communications internes et externes tout au long de l'incident.
+Le groupe F24 compte 5500 clients à travers le monde dont 30% des acteurs du CAC40.</t>
+        </is>
+      </c>
+      <c r="E285" s="3" t="inlineStr"/>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA : Gestion des incidents
+RC.CO : Communication de la reprise
+GV.RM : Stratégie de gestion des risques</t>
+        </is>
+      </c>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA-01 : Le plan de réponse aux incidents est exécuté en coordination avec les tiers concernés
+RC.CO-03 : Les activités et l'avancement de la reprise sont communiqués aux parties prenantes désignées
+RC.CO-04 : Les communications publiques sur la reprise d'incident utilisent des méthodes et messages approuvés</t>
+        </is>
+      </c>
+      <c r="I285" s="3" t="inlineStr">
+        <is>
+          <t>Continuité et reprise d'activité</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>https://f24.com/fr/produits/solutions-notification-urgence-gestion-de-crise/</t>
+        </is>
+      </c>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>Arnaud.sraka@f24.com</t>
+        </is>
+      </c>
+      <c r="L285" s="2" t="inlineStr">
+        <is>
+          <t>f24.png</t>
+        </is>
+      </c>
+      <c r="M285" s="2" t="inlineStr">
+        <is>
+          <t>f24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M284"/>
+  <autoFilter ref="A1:M285"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24866,7 +24936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J284"/>
+  <dimension ref="A1:J285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38861,8 +38931,44 @@
       <c r="I284" s="3" t="inlineStr"/>
       <c r="J284" s="3" t="inlineStr"/>
     </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>RS : Répondre</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA : Gestion des incidents
+RC.CO : Communication de la reprise
+GV.RM : Stratégie de gestion des risques</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>RS.MA-01 : Le plan de réponse aux incidents est exécuté en coordination avec les tiers concernés
+RC.CO-03 : Les activités et l'avancement de la reprise sont communiqués aux parties prenantes désignées
+RC.CO-04 : Les communications publiques sur la reprise d'incident utilisent des méthodes et messages approuvés</t>
+        </is>
+      </c>
+      <c r="E285" s="3" t="inlineStr"/>
+      <c r="F285" s="3" t="inlineStr"/>
+      <c r="G285" s="3" t="inlineStr"/>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>Grand groupe</t>
+        </is>
+      </c>
+      <c r="I285" s="3" t="inlineStr"/>
+      <c r="J285" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J284"/>
+  <autoFilter ref="A1:J285"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #150 : Advens [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Classement &amp; justification" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$285</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$285</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Solutions'!$A$1:$M$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Classement &amp; justification'!$A$1:$J$286</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M285"/>
+  <dimension ref="A1:M286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -19678,8 +19678,75 @@
         </is>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Advens</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>ETI / scale-up</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>VulSight, édité par Advens, est une plateforme unifiée de gestion des vulnérabilités qui centralise les données issues de multiples solutions de sécurité (Qualys, Tenable, Wiz, CrowdStrike, etc.) afin d’offrir une vision consolidée de l’exposition aux risques. Grâce à des mécanismes de priorisation assistés par l’IA et à l’enrichissement des données par des référentiels tels que CISA KEV et EPSS, VulSight aide les organisations à concentrer leurs efforts de remédiation sur les vulnérabilités les plus critiques et à accélérer leur traitement.</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>VulSight aide les organisations à reprendre le contrôle de leur exposition aux vulnérabilités en centralisant les informations provenant de leurs différents outils de sécurité au sein d’une plateforme unique. La solution offre une vision consolidée des risques, facilite leur priorisation et permet aux équipes de se concentrer sur les actions de remédiation les plus pertinentes.
+En fournissant un contexte enrichi sur les vulnérabilités et leur exploitabilité, VulSight simplifie la prise de décision et améliore l’efficacité des programmes de gestion des vulnérabilités. Les organisations peuvent ainsi réduire plus rapidement leur surface d’exposition tout en optimisant les efforts de leurs équipes cyber.</t>
+        </is>
+      </c>
+      <c r="E286" s="3" t="inlineStr"/>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>ID : Identifier</t>
+        </is>
+      </c>
+      <c r="G286" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA : Évaluation des risques
+DE.CM : Surveillance continue</t>
+        </is>
+      </c>
+      <c r="H286" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA-01 : Les vulnérabilités des actifs sont identifiées, validées et enregistrées
+ID.RA-04 : Les impacts et probabilités potentiels des menaces exploitant les vulnérabilités sont enregistrés
+DE.CM-09 : Le matériel, les logiciels et les environnements d'exécution sont surveillés pour détecter les événements indésirables</t>
+        </is>
+      </c>
+      <c r="I286" s="3" t="inlineStr">
+        <is>
+          <t>Maîtrise des SI</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>https://advens.com/</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>contact@advens.fr</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>advens.png</t>
+        </is>
+      </c>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>advens</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M285"/>
+  <autoFilter ref="A1:M286"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24936,7 +25003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J285"/>
+  <dimension ref="A1:J286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38967,8 +39034,43 @@
       <c r="I285" s="3" t="inlineStr"/>
       <c r="J285" s="3" t="inlineStr"/>
     </row>
+    <row r="286">
+      <c r="A286" s="3" t="inlineStr">
+        <is>
+          <t>Advens</t>
+        </is>
+      </c>
+      <c r="B286" s="3" t="inlineStr">
+        <is>
+          <t>ID : Identifier</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA : Évaluation des risques
+DE.CM : Surveillance continue</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>ID.RA-01 : Les vulnérabilités des actifs sont identifiées, validées et enregistrées
+ID.RA-04 : Les impacts et probabilités potentiels des menaces exploitant les vulnérabilités sont enregistrés
+DE.CM-09 : Le matériel, les logiciels et les environnements d'exécution sont surveillés pour détecter les événements indésirables</t>
+        </is>
+      </c>
+      <c r="E286" s="3" t="inlineStr"/>
+      <c r="F286" s="3" t="inlineStr"/>
+      <c r="G286" s="3" t="inlineStr"/>
+      <c r="H286" s="3" t="inlineStr">
+        <is>
+          <t>ETI / scale-up</t>
+        </is>
+      </c>
+      <c r="I286" s="3" t="inlineStr"/>
+      <c r="J286" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J285"/>
+  <autoFilter ref="A1:J286"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Soumission #151 : Tenacy [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -15771,12 +15771,12 @@
       </c>
       <c r="K227" s="2" t="inlineStr">
         <is>
-          <t>contact@tenacy.io</t>
+          <t>corentin.mirande@tenacy.io</t>
         </is>
       </c>
       <c r="L227" s="2" t="inlineStr">
         <is>
-          <t>Tenacy_svg.svg</t>
+          <t>tenacy.png</t>
         </is>
       </c>
       <c r="M227" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Soumission #152 : SNOWPACK [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -15040,8 +15040,8 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>**Fournisseur de connectivité furtive, sécurisée et résiliente.** 
-Grâce à notre technologie brevetée VIPN (_Virtual &amp; Invisible Private Network_), réduisez et protégez votre surface d’attaque externe en ne faisant confiance à personne: rendez **invisibles** vos assets numériques sensibles exposés sur Internet et protégez vos utilisateurs, services et infrastructures des cyberattaques.</t>
+          <t>Fournisseur de connectivité furtive, sécurisée et résiliente.
+Grâce à notre technologie brevetée VIPN (Virtual &amp; Invisible Private Network), réduisez et protégez votre surface d’attaque externe en ne faisant confiance à personne: rendez invisibles vos assets numériques sensibles exposés sur Internet et protégez vos utilisateurs, services et infrastructures des cyberattaques.</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Soumission #154 : Gatewatcher (NDR Gatewatcher) [approved]
</commit_message>
<xml_diff>
--- a/data/solutions_master.xlsx
+++ b/data/solutions_master.xlsx
@@ -6886,7 +6886,7 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Gatewatcher conçoit une plateforme de détection et de réponse réseau (NDR) qui surveille les flux et les actifs pour repérer les menaces. La solution réunit les capteurs Sensor et TAP, le moteur Deep Visibility et le Decision Center qui priorise les alertes et accélère le triage. Parmi ses clients figurent la Banque de France, BNP Paribas, Sanofi, EDF, le CNES, Dassault et Naval Group, dans la finance, l'industrie, la défense, la santé et le secteur public.</t>
+          <t>Gatewatcher commercialise une plateforme de cybersécurité combinant NDR et Decision Center pour transformer les signaux de sécurité en décisions directement exploitables. Son NDR apporte une visibilité approfondie sur les flux, les actifs et les comportements réseau afin de détecter les menaces, tandis que Decision Center, fondé sur une approche d’IA agentique, corrèle les alertes issues du réseau et des autres outils du SOC pour produire des décisions contextualisées, explicables et actionnables. Gatewatcher accompagne notamment des organisations telles que la Banque de France, BNP Paribas, Sanofi, EDF, le CNES, Dassault et Naval Group dans les secteurs de la finance, de l’industrie, de la défense, de la santé et du secteur public.</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -6911,10 +6911,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables
-DE.CM-02 : L'environnement physique est surveillé pour détecter les événements potentiellement indésirables
-DE.CM-06 : Les activités et services des prestataires externes sont surveillés pour détecter les événements indésirables
-DE.CM-09 : Le matériel, les logiciels et les environnements d'exécution sont surveillés pour détecter les événements indésirables</t>
+          <t>DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -29754,10 +29751,7 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables
-DE.CM-02 : L'environnement physique est surveillé pour détecter les événements potentiellement indésirables
-DE.CM-06 : Les activités et services des prestataires externes sont surveillés pour détecter les événements indésirables
-DE.CM-09 : Le matériel, les logiciels et les environnements d'exécution sont surveillés pour détecter les événements indésirables</t>
+          <t>DE.CM-01 : Les réseaux et services réseau sont surveillés pour détecter les événements potentiellement indésirables</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">

</xml_diff>